<commit_message>
Add phone numbers for 11 of 13 missing companies
Found via web scraping: Izrastzoff, Rapaport, Llauro, Soldati,
LJ Ramos, Toribio Achával, Miranda Bosch, Korn, Mudafy, ATV
Arquitectos, Grupo Upgrade. Also corrected web domains (izr.com.ar,
rapaport.ar, soldati.com, toribioachaval.com). Only Grow Desarrollos
(no BA presence) and Nova Desarrollos (no public phone) remain without.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LfLhTAy3dmahxAx9Ya2Hd9
</commit_message>
<xml_diff>
--- a/Desarrollistas_Inmobiliarias_BA_Integrado.xlsx
+++ b/Desarrollistas_Inmobiliarias_BA_Integrado.xlsx
@@ -1138,7 +1138,11 @@
           <t>Desarrollista Boutique</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>+54 11 4890-7070 / WA: +54 11 4096-0600</t>
+        </is>
+      </c>
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr">
         <is>
@@ -1454,7 +1458,11 @@
           <t>Desarrollista Boutique</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>+54 11 2167-4070</t>
+        </is>
+      </c>
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="2" t="inlineStr">
         <is>
@@ -2814,11 +2822,15 @@
           <t>Inmobiliaria Premium</t>
         </is>
       </c>
-      <c r="C41" s="3" t="inlineStr"/>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>+54 11 5279-1001 / WA: +54 9 11 3830-9311</t>
+        </is>
+      </c>
       <c r="D41" s="3" t="inlineStr"/>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>izrastzoff.com.ar</t>
+          <t>izr.com.ar</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr"/>
@@ -2860,11 +2872,15 @@
           <t>Inmobiliaria Premium</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr"/>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>+54 9 11 5369-7887 (WA)</t>
+        </is>
+      </c>
       <c r="D42" s="3" t="inlineStr"/>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>rapaport.com.ar</t>
+          <t>rapaport.ar</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr"/>
@@ -2908,7 +2924,7 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>4816-8000</t>
+          <t>+54 11 4816-8000 / WA: +54 9 11 4047-1616</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr"/>
@@ -2956,11 +2972,15 @@
           <t>Inmobiliaria Premium</t>
         </is>
       </c>
-      <c r="C44" s="3" t="inlineStr"/>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>+54 9 11 7700-1010</t>
+        </is>
+      </c>
       <c r="D44" s="3" t="inlineStr"/>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>soldati.com.ar</t>
+          <t>soldati.com</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr"/>
@@ -3002,11 +3022,15 @@
           <t>Inmobiliaria Premium</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr"/>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>+54 11 4114-1000 / WA: +54 9 11 4114-1000</t>
+        </is>
+      </c>
       <c r="D45" s="3" t="inlineStr"/>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>ljramos.com.ar</t>
+          <t>ljramos.com</t>
         </is>
       </c>
       <c r="F45" s="3" t="inlineStr"/>
@@ -3048,11 +3072,15 @@
           <t>Inmobiliaria Premium</t>
         </is>
       </c>
-      <c r="C46" s="3" t="inlineStr"/>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>+54 11 4819-4000 / WA: +54 9 11 6525-6809</t>
+        </is>
+      </c>
       <c r="D46" s="3" t="inlineStr"/>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>toribioachával.com</t>
+          <t>toribioachaval.com</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr"/>
@@ -3094,7 +3122,11 @@
           <t>Inmobiliaria Premium</t>
         </is>
       </c>
-      <c r="C47" s="3" t="inlineStr"/>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>+54 11 4815-3515 / WA: +54 9 11 2305-9696</t>
+        </is>
+      </c>
       <c r="D47" s="3" t="inlineStr"/>
       <c r="E47" s="3" t="inlineStr">
         <is>
@@ -3140,7 +3172,11 @@
           <t>Inmobiliaria Premium</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr"/>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>+54 9 11 7856-7071 / 0810-444-5676</t>
+        </is>
+      </c>
       <c r="D48" s="3" t="inlineStr"/>
       <c r="E48" s="3" t="inlineStr">
         <is>
@@ -3186,7 +3222,11 @@
           <t>Inmobiliaria Premium</t>
         </is>
       </c>
-      <c r="C49" s="3" t="inlineStr"/>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>+54 9 11 6730-8230 (WA)</t>
+        </is>
+      </c>
       <c r="D49" s="3" t="inlineStr"/>
       <c r="E49" s="3" t="inlineStr">
         <is>

</xml_diff>